<commit_message>
BIS-2697: Fixed export tests
</commit_message>
<xml_diff>
--- a/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-sample-cell-with-images.xlsx
+++ b/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-sample-cell-with-images.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">SAMPLE</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">Modification Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meta Data</t>
   </si>
   <si>
     <t xml:space="preserve">Name</t>
@@ -311,119 +314,13 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMM5"/>
-  <sheetFormatPr defaultColWidth="10.51171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Q5"/>
+  <sheetFormatPr defaultColWidth="10.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.5"/>
@@ -436,9 +333,6 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="1025" style="1" width="8.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16383" min="16382" style="1" width="8.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="9.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -503,60 +397,60 @@
       <c r="M4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="9"/>
-      <c r="AML4" s="1"/>
-      <c r="AMM4" s="1"/>
+      <c r="P4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="11"/>
       <c r="I5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="13" t="s">
         <v>28</v>
       </c>
+      <c r="M5" s="12"/>
       <c r="N5" s="13" t="s">
         <v>29</v>
       </c>
       <c r="O5" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="AML5" s="1"/>
-      <c r="AMM5" s="1"/>
+      <c r="P5" s="13" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>